<commit_message>
add greenhouse conditions and variance partition to CO2 partitioning
- CO2_partitioning_by_occasion: rows for greenhouse temperature, PAR and
  relative humidity under the GPP/ER/NEE panels, per treatment
- variance_partition sheet: variance in GPP, ER and NEE explained by
  occasion after correcting for temperature, PAR and humidity (linear
  models, plus a mixed model with pot as random intercept)
- regenerate outputs
</commit_message>
<xml_diff>
--- a/output/tables/CO2_partitioning.xlsx
+++ b/output/tables/CO2_partitioning.xlsx
@@ -12,6 +12,7 @@
     <sheet name="totals_per_pot" sheetId="3" r:id="rId3"/>
     <sheet name="totals_means" sheetId="4" r:id="rId4"/>
     <sheet name="totals_pairwise" sheetId="5" r:id="rId5"/>
+    <sheet name="variance_partition" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -37030,4 +37031,272 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:Q4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>environment_window</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>R2_occasion_alone</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>R2_environment_alone</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>dR2_occasion_after_environment</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>dR2_occasion_after_environment_treatment_block</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>dR2_environment_after_occasion_treatment_block</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>dR2_treatment_after_environment_occasion_block</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>R2_full</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>mixed_pot_variance</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>mixed_residual_variance</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>mixed_marginal_R2_full</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>mixed_dR2m_occasion</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>mixed_LRT_chisq_occasion</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>mixed_LRT_df</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>mixed_LRT_p_occasion</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>NEE</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>358</v>
+      </c>
+      <c r="D2">
+        <v>0.4011635070284504</v>
+      </c>
+      <c r="E2">
+        <v>0.07192760313916148</v>
+      </c>
+      <c r="F2">
+        <v>0.3720682905565728</v>
+      </c>
+      <c r="G2">
+        <v>0.3810477682930289</v>
+      </c>
+      <c r="H2">
+        <v>0.001103951896359034</v>
+      </c>
+      <c r="I2">
+        <v>0.179971065195443</v>
+      </c>
+      <c r="J2">
+        <v>0.6856880282753393</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2">
+        <v>0.2097815200133294</v>
+      </c>
+      <c r="M2">
+        <v>0.686290568335981</v>
+      </c>
+      <c r="N2">
+        <v>0.3810574401171246</v>
+      </c>
+      <c r="O2">
+        <v>284.2674978158684</v>
+      </c>
+      <c r="P2">
+        <v>14</v>
+      </c>
+      <c r="Q2">
+        <v>2.236355579030938E-52</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ER</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Dark</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>357</v>
+      </c>
+      <c r="D3">
+        <v>0.3788748452290757</v>
+      </c>
+      <c r="E3">
+        <v>0.2483482236965899</v>
+      </c>
+      <c r="F3">
+        <v>0.2583899379853385</v>
+      </c>
+      <c r="G3">
+        <v>0.2871238583988016</v>
+      </c>
+      <c r="H3">
+        <v>0.01013839995018551</v>
+      </c>
+      <c r="I3">
+        <v>0.1741755670269216</v>
+      </c>
+      <c r="J3">
+        <v>0.7262261473052137</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3">
+        <v>0.03082431031255759</v>
+      </c>
+      <c r="M3">
+        <v>0.7267834983371882</v>
+      </c>
+      <c r="N3">
+        <v>0.2869902317372528</v>
+      </c>
+      <c r="O3">
+        <v>256.053303859604</v>
+      </c>
+      <c r="P3">
+        <v>14</v>
+      </c>
+      <c r="Q3">
+        <v>1.606478903875984E-46</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>GPP</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>357</v>
+      </c>
+      <c r="D4">
+        <v>0.4116416666406013</v>
+      </c>
+      <c r="E4">
+        <v>0.1295271077225101</v>
+      </c>
+      <c r="F4">
+        <v>0.3540922500128746</v>
+      </c>
+      <c r="G4">
+        <v>0.3683628009532126</v>
+      </c>
+      <c r="H4">
+        <v>0.003443420019924481</v>
+      </c>
+      <c r="I4">
+        <v>0.1898000337441452</v>
+      </c>
+      <c r="J4">
+        <v>0.7333713919761364</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>0.3139410808286572</v>
+      </c>
+      <c r="M4">
+        <v>0.7339195262665853</v>
+      </c>
+      <c r="N4">
+        <v>0.3682605422086602</v>
+      </c>
+      <c r="O4">
+        <v>309.7884495796687</v>
+      </c>
+      <c r="P4">
+        <v>14</v>
+      </c>
+      <c r="Q4">
+        <v>1.072045477415067E-57</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>